<commit_message>
added indicator descriptions to excel report
</commit_message>
<xml_diff>
--- a/backend/State of the Market Report - Oct 2023.xlsx
+++ b/backend/State of the Market Report - Oct 2023.xlsx
@@ -5,13 +5,14 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Indicator - MoM Comparison" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Indicator Descriptions" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="34">
   <si>
     <t>Indicator</t>
   </si>
@@ -77,6 +78,42 @@
   </si>
   <si>
     <t>Consumer Confidence</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>10-year yield estimated from the average yields of a variety of Treasury securities with different maturities derived from the Treasury yield curve.</t>
+  </si>
+  <si>
+    <t>Effective Federal Funds Rate, or the interest rate depository institutions charge each other for overnight loans of funds.</t>
+  </si>
+  <si>
+    <t>A benchmark of average single-family home prices in the U.S., calculated monthly based on changes in home prices over the prior three months.</t>
+  </si>
+  <si>
+    <t>The number of people 16 and over actively searching for a job as a percentage of the total labor force.</t>
+  </si>
+  <si>
+    <t>An inflation measure derived from tracking the changes in the weighted-average price of a basket of common goods and services.</t>
+  </si>
+  <si>
+    <t>An index that measures monthly changes in the price of consumer goods and services as a means of analyzing inflation.</t>
+  </si>
+  <si>
+    <t>A measure of all jobs that are not filled on the last business day of the month. A job is considered open if a specific position exists and there is work available for it, the job can be started within 30 days, and there is active recruiting for the position.</t>
+  </si>
+  <si>
+    <t>Workers hired</t>
+  </si>
+  <si>
+    <t>Workers that quit their job, were laid off, or experienced other separations (including worker deaths)</t>
+  </si>
+  <si>
+    <t>Personal saving as a percentage of disposable personal income (DPI), frequently referred to as "the personal saving rate," is calculated as the ratio of personal saving to DPI. Personal saving is equal to personal income less personal outlays and personal taxes; it may generally be viewed as the portion of personal income that is used either to provide funds to capital markets or to invest in real assets such as residences.</t>
+  </si>
+  <si>
+    <t>Provides an indication of future developments of households' consumption and saving, based upon answers regarding their expected financial situation, their sentiment about the general economic situation, unemployment and capability of savings.</t>
   </si>
 </sst>
 </file>
@@ -709,4 +746,114 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="2" width="9" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>